<commit_message>
Clean up Memory Aids
</commit_message>
<xml_diff>
--- a/Models/SA1_Assumption_Setting_Model.xlsx
+++ b/Models/SA1_Assumption_Setting_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Girish\IAI\SP1 and SA1 Health and Care\Practice papers\Claude Widgets\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70710E68-12BD-4538-97BC-E6E9A23D1B1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75EE42B-C069-4738-831A-21D0AE366B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -1011,7 +1011,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1058,11 +1058,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBDD7EE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1129,13 +1138,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1147,6 +1151,16 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1607,7 +1621,7 @@
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="5" max="5" width="42.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1746,12 +1760,12 @@
     </row>
     <row r="12" spans="2:5" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
@@ -1774,7 +1788,6 @@
       <c r="D15" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="24"/>
     </row>
     <row r="16" spans="2:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11" t="s">
@@ -1786,7 +1799,6 @@
       <c r="D16" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="25"/>
     </row>
     <row r="17" spans="2:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="14" t="s">
@@ -1798,7 +1810,6 @@
       <c r="D17" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E17" s="24"/>
     </row>
     <row r="18" spans="2:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="11" t="s">
@@ -1810,26 +1821,21 @@
       <c r="D18" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="25"/>
     </row>
     <row r="20" spans="2:5" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="2:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="3">
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="E17"/>
-    <mergeCell ref="E18"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="E15"/>
-    <mergeCell ref="E16"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B21:D21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2272,7 +2278,7 @@
       </c>
     </row>
     <row r="17" spans="2:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="24" t="s">
         <v>163</v>
       </c>
       <c r="C17" s="20"/>
@@ -2368,13 +2374,13 @@
     </row>
     <row r="6" spans="2:6" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="2:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
     </row>
     <row r="8" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
@@ -2392,7 +2398,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="10" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>185</v>
       </c>
@@ -2426,8 +2432,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B7:F7"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2456,7 +2462,7 @@
       <c r="F1" s="20"/>
     </row>
     <row r="2" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="29" t="s">
         <v>194</v>
       </c>
       <c r="C2" s="20"/>
@@ -2610,7 +2616,7 @@
     </row>
     <row r="14" spans="2:6" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="29" t="s">
         <v>226</v>
       </c>
       <c r="C15" s="20"/>
@@ -2695,7 +2701,7 @@
     </row>
     <row r="22" spans="2:6" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="29" t="s">
         <v>244</v>
       </c>
       <c r="C23" s="20"/>
@@ -2704,81 +2710,81 @@
       <c r="F23" s="20"/>
     </row>
     <row r="24" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="27"/>
       <c r="F24" s="10"/>
     </row>
     <row r="25" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="13" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="27"/>
       <c r="F26" s="10" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="30"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="27"/>
       <c r="F27" s="13" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="25" t="s">
         <v>251</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="30"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="27"/>
       <c r="F28" s="10" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="28" t="s">
         <v>253</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="30"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="13" t="s">
         <v>203</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B24:E24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2944,7 +2950,7 @@
       </c>
     </row>
     <row r="13" spans="2:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="24" t="s">
         <v>284</v>
       </c>
       <c r="C13" s="20"/>

</xml_diff>